<commit_message>
Added HP roll-off characteristics.
</commit_message>
<xml_diff>
--- a/RIAAResponse/StateVarResponse.xlsx
+++ b/RIAAResponse/StateVarResponse.xlsx
@@ -4,12 +4,18 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28125"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="160" windowWidth="25600" windowHeight="18380" tabRatio="500"/>
+    <workbookView xWindow="39460" yWindow="1540" windowWidth="25600" windowHeight="18380" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Measured RIAA Response" sheetId="1" r:id="rId1"/>
     <sheet name="RIAADeemphasisChart" sheetId="2" r:id="rId2"/>
+    <sheet name="LowFreqRollOffs" sheetId="3" r:id="rId3"/>
+    <sheet name="HPRolloffChart" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_t4">LowFreqRollOffs!$D$4</definedName>
+    <definedName name="_t5">LowFreqRollOffs!$D$5</definedName>
+  </definedNames>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
@@ -20,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="56">
   <si>
     <t>Loading</t>
   </si>
@@ -132,11 +138,71 @@
   <si>
     <t>Frequency</t>
   </si>
+  <si>
+    <t>diff</t>
+  </si>
+  <si>
+    <t>min:</t>
+  </si>
+  <si>
+    <t>max:</t>
+  </si>
+  <si>
+    <t>delta:</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t>Omega</t>
+  </si>
+  <si>
+    <t>First</t>
+  </si>
+  <si>
+    <t>Second</t>
+  </si>
+  <si>
+    <t>XferFcn</t>
+  </si>
+  <si>
+    <t>Combined</t>
+  </si>
+  <si>
+    <t>Gain</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Normalized</t>
+  </si>
+  <si>
+    <t>Gain (dB)</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Const (sec)</t>
+  </si>
+  <si>
+    <t>Servo bias circuit</t>
+  </si>
+  <si>
+    <t>DC blocking capacitor at input</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -187,22 +253,33 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="9">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -249,7 +326,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -1888,11 +1964,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-2141846616"/>
-        <c:axId val="2136739944"/>
+        <c:axId val="2129949144"/>
+        <c:axId val="2129952280"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="-2141846616"/>
+        <c:axId val="2129949144"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -1917,12 +1993,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2136739944"/>
+        <c:crossAx val="2129952280"/>
         <c:crossesAt val="-35.0"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2136739944"/>
+        <c:axId val="2129952280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="140.0"/>
@@ -1945,7 +2021,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2141846616"/>
+        <c:crossAx val="2129949144"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="25.0"/>
@@ -1953,7 +2029,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:txPr>
         <a:bodyPr/>
@@ -2022,7 +2097,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -2897,8 +2971,8 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-2140711992"/>
-        <c:axId val="-2140619368"/>
+        <c:axId val="2130041416"/>
+        <c:axId val="2130044440"/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
@@ -3225,7 +3299,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Measured RIAA Response'!$T$80:$T$110</c:f>
+              <c:f>'Measured RIAA Response'!$S$80:$S$110</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
@@ -3335,11 +3409,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-2143079272"/>
-        <c:axId val="-2141229688"/>
+        <c:axId val="2130050520"/>
+        <c:axId val="2130047480"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="-2140711992"/>
+        <c:axId val="2130041416"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -3364,12 +3438,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2140619368"/>
+        <c:crossAx val="2130044440"/>
         <c:crossesAt val="-160.0"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2140619368"/>
+        <c:axId val="2130044440"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3390,12 +3464,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2140711992"/>
+        <c:crossAx val="2130041416"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2141229688"/>
+        <c:axId val="2130047480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3405,12 +3479,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2143079272"/>
+        <c:crossAx val="2130050520"/>
         <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2143079272"/>
+        <c:axId val="2130050520"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -3433,14 +3507,13 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2141229688"/>
+        <c:crossAx val="2130047480"/>
         <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:txPr>
         <a:bodyPr/>
@@ -3955,8 +4028,8 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-2136271464"/>
-        <c:axId val="-2136566696"/>
+        <c:axId val="2130302888"/>
+        <c:axId val="2130308648"/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
@@ -4283,7 +4356,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Measured RIAA Response'!$T$80:$T$110</c:f>
+              <c:f>'Measured RIAA Response'!$S$80:$S$110</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
@@ -4393,11 +4466,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-2138071656"/>
-        <c:axId val="-2138474824"/>
+        <c:axId val="2130319544"/>
+        <c:axId val="2130314072"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="-2136271464"/>
+        <c:axId val="2130302888"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -4441,12 +4514,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2136566696"/>
+        <c:crossAx val="2130308648"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2136566696"/>
+        <c:axId val="2130308648"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.9"/>
@@ -4489,14 +4562,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2136271464"/>
+        <c:crossAx val="2130302888"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.1"/>
         <c:minorUnit val="0.025"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2138474824"/>
+        <c:axId val="2130314072"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="20.0"/>
@@ -4544,13 +4617,13 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2138071656"/>
+        <c:crossAx val="2130319544"/>
         <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="4.0"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2138071656"/>
+        <c:axId val="2130319544"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -4573,7 +4646,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2138474824"/>
+        <c:crossAx val="2130314072"/>
         <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4600,7 +4673,1624 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="118"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="18"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>RIAA Response With Servo and DC Block</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>6 June 2026</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.0954099182724111"/>
+          <c:y val="0.161360391175593"/>
+          <c:w val="0.809833877472633"/>
+          <c:h val="0.69196561710573"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>HP Phase (deg)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400"/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>LowFreqRollOffs!$C$9:$C$39</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>16.001451</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20.143118</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>25.362768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31.929302</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.195312</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.597405</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>63.69847</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>80.201261</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>100.968027</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>127.10439</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>160.007022</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>201.456349</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>253.585211</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>319.290075</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>401.94414</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>506.015299</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>636.97723</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>801.911445</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1009.546788</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1271.06546</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1600.019278</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2014.313892</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2536.107678</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3192.521598</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4019.460315</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5059.790831</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>6369.735421</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8019.263685</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>10096.471541</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12710.556156</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>16000.960204</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>LowFreqRollOffs!$I$9:$I$39</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>16.2779489711051</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12.97328820950548</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.32484657752718</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.212278162698142</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.528905908039324</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.189397359772232</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.123454256417914</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.275673466852456</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.602290245880616</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.067357245291046</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.64232862568104</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.304465759564095</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.036331945158887</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.823082140925451</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.653832562781412</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.519362876167984</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.412583728217859</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.327725707191702</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.260322105683197</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.2067616302664</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.164252837232111</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.130470129335503</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.103626455538771</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.082319845449711</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.0653838789412262</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.0519404713275961</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.0412588454633406</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.0327720779926931</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.0260296814946349</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.0206763525856463</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.0164245106971291</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Left Phase (deg)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="triangle"/>
+            <c:size val="6"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Measured RIAA Response'!$I$80:$I$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>16.001451</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20.143118</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>25.362768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31.929302</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.195312</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.597405</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>63.69847</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>80.201261</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>100.968027</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>127.10439</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>160.007022</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>201.456349</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>253.585211</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>319.290075</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>401.94414</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>506.015299</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>636.97723</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>801.911445</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1009.546788</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1271.06546</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1600.019278</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2014.313892</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2536.107678</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3192.521598</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4019.460315</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5059.790831</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>6369.735421</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8019.263685</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>10096.471541</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12710.556156</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>16000.960204</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Measured RIAA Response'!$R$80:$R$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>15.20728701074722</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12.1106102142958</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.636896557823806</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.665633604061593</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.096761544089225</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.851630505697932</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.847329190270898</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.050928920334176</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.414886214079478</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.899959357398448</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.487147142460425</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.150792641148981</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.87619297100963</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.648632934707852</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.456512946056912</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.293222674937846</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.154068548309159</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.0315800476626854</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-0.07320405624315</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-0.169459260595185</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>-0.247752701602752</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>-0.31128933671961</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>-0.363695894006923</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-0.408677861308783</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>-0.453645873299276</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-0.504550879904461</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-0.577427731243562</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>-0.680585766806826</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>-0.79578839642323</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>-0.97398087826191</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>-1.190295722902536</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:v>Right Phase (deg)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="6"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Measured RIAA Response'!$I$80:$I$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>16.001451</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20.143118</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>25.362768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31.929302</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.195312</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.597405</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>63.69847</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>80.201261</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>100.968027</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>127.10439</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>160.007022</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>201.456349</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>253.585211</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>319.290075</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>401.94414</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>506.015299</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>636.97723</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>801.911445</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1009.546788</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1271.06546</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1600.019278</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2014.313892</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2536.107678</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3192.521598</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4019.460315</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5059.790831</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>6369.735421</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8019.263685</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>10096.471541</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12710.556156</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>16000.960204</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Measured RIAA Response'!$S$80:$S$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>15.95312384993777</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12.7138322080614</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.11191160605383</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.034146932019838</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.386773006061015</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.061883076270845</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.025943991665574</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.197007721159731</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.533828359572577</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.007806245110845</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.585084682859773</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.243990176134715</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.967375656893329</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.742425549458988</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.556425487119562</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.402551114698366</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.274606643814133</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.16706651012608</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.0749467860712682</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-0.00503396790610215</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>-0.0742417397140494</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>-0.135578859935961</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>-0.196234532767246</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-0.257828884559367</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>-0.326980734544899</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-0.408134146520791</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-0.512619431828231</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>-0.648813767460889</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>-0.79810117785488</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>-1.012078553004088</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>-1.267139428473298</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="2130389880"/>
+        <c:axId val="2130392872"/>
+      </c:scatterChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>HP Gain (dB)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400"/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>LowFreqRollOffs!$C$9:$C$39</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>16.001451</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20.143118</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>25.362768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31.929302</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.195312</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.597405</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>63.69847</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>80.201261</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>100.968027</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>127.10439</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>160.007022</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>201.456349</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>253.585211</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>319.290075</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>401.94414</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>506.015299</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>636.97723</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>801.911445</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1009.546788</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1271.06546</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1600.019278</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2014.313892</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2536.107678</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3192.521598</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4019.460315</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5059.790831</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>6369.735421</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8019.263685</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>10096.471541</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12710.556156</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>16000.960204</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>LowFreqRollOffs!$J$9:$J$39</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>1.605248298408453</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.676418740256666</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.721774912159264</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.750531053189306</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.768740910430426</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.780254874541198</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.787534649633868</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.792133970203398</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.795035810596327</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.796867025289502</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.798022852905047</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.79875267444337</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.799212755838367</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.79950341193099</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.799686641189202</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.799802280307038</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.799875223766232</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.799921272144501</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.79995032597806</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.799968663750758</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.799980224257085</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1.799987522453721</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1.799992128667416</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1.799995032749637</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.799996866365713</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.799998022489892</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1.799998752211219</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.799999212745971</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1.799999503356629</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1.799999686631897</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1.799999802261235</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Left Gain (dB)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Measured RIAA Response'!$I$80:$I$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>16.001451</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20.143118</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>25.362768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31.929302</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.195312</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.597405</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>63.69847</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>80.201261</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>100.968027</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>127.10439</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>160.007022</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>201.456349</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>253.585211</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>319.290075</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>401.94414</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>506.015299</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>636.97723</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>801.911445</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1009.546788</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1271.06546</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1600.019278</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2014.313892</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2536.107678</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3192.521598</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4019.460315</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5059.790831</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>6369.735421</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8019.263685</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>10096.471541</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12710.556156</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>16000.960204</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Measured RIAA Response'!$N$80:$N$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>1.64460791769961</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.70515486083573</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.745079063089538</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.769799866341</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.786068852592347</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.797588512908772</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.805250246014604</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.81094249115254</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.814328035049075</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.817577729116179</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.819754058600674</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.821639729538111</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.822454673873817</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.822526403219069</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.822406844395464</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.82023957074668</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.818055054583497</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.812939717707637</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.80832507875774</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.801571815350778</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.793645567667261</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1.785456624690366</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1.777730463092631</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1.771573638795289</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.764481531394602</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.762670877181318</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1.7583818830354</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.756933326497492</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1.757339349676366</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1.756728471342165</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1.757836056482555</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Right Gain (dB)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="square"/>
+            <c:size val="6"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Measured RIAA Response'!$I$80:$I$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>16.001451</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20.143118</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>25.362768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31.929302</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.195312</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.597405</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>63.69847</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>80.201261</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>100.968027</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>127.10439</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>160.007022</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>201.456349</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>253.585211</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>319.290075</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>401.94414</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>506.015299</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>636.97723</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>801.911445</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1009.546788</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1271.06546</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1600.019278</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2014.313892</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2536.107678</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3192.521598</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4019.460315</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5059.790831</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>6369.735421</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8019.263685</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>10096.471541</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12710.556156</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>16000.960204</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Measured RIAA Response'!$P$80:$P$110</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>1.613179625170913</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.680964062187866</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.72622794414578</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.752543899609704</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.77014816706576</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.783812131098279</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.78926623078071</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.794055330760887</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.797213983467848</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.800212385611787</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.802385123139063</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.804672263376564</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.80613096930524</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.807067759835581</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.807801755321815</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.807677492107896</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.80704416355398</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.80487105524783</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.803270609981024</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.800688193560065</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.798126153723766</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1.796039576330928</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1.794903937656121</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1.794169691043119</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.79379831678353</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.793063629992384</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1.793405455966681</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.794170518611799</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1.79639214787529</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1.797375894357351</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1.800149697466653</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="2130399176"/>
+        <c:axId val="2130396184"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="2130389880"/>
+        <c:scaling>
+          <c:logBase val="10.0"/>
+          <c:orientation val="minMax"/>
+          <c:max val="16000.0"/>
+          <c:min val="16.0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines/>
+        <c:minorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Frequency</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> (Hz)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.45343573052904"/>
+              <c:y val="0.882686823832571"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="cross"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2130392872"/>
+        <c:crossesAt val="-4.0"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="2130392872"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="20.0"/>
+          <c:min val="-4.0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400"/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Phase (deg)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="cross"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2130389880"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="4.0"/>
+        <c:minorUnit val="1.0"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="2130396184"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1.9"/>
+          <c:min val="1.3"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:minorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400"/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Gain (dB)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="cross"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2130399176"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+        <c:minorUnit val="0.025"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="2130399176"/>
+        <c:scaling>
+          <c:logBase val="10.0"/>
+          <c:orientation val="minMax"/>
+          <c:max val="16000.0"/>
+          <c:min val="16.0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="t"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2130396184"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
 <file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
+<file path=xl/chartsheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4650,8 +6340,8 @@
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>112</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4674,6 +6364,33 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="9209497" cy="5623145"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
@@ -5022,7 +6739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U110"/>
+  <dimension ref="A1:T114"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -8359,7 +10076,7 @@
         <v>11.712447757474006</v>
       </c>
     </row>
-    <row r="65" spans="1:21">
+    <row r="65" spans="1:20">
       <c r="A65">
         <v>2014.3138919999999</v>
       </c>
@@ -8420,7 +10137,7 @@
         <v>14.091552726061041</v>
       </c>
     </row>
-    <row r="66" spans="1:21">
+    <row r="66" spans="1:20">
       <c r="A66">
         <v>2536.1076779999999</v>
       </c>
@@ -8481,7 +10198,7 @@
         <v>20.011534503038963</v>
       </c>
     </row>
-    <row r="67" spans="1:21">
+    <row r="67" spans="1:20">
       <c r="A67">
         <v>3192.5215979999998</v>
       </c>
@@ -8542,7 +10259,7 @@
         <v>16.929219795181204</v>
       </c>
     </row>
-    <row r="68" spans="1:21">
+    <row r="68" spans="1:20">
       <c r="A68">
         <v>4019.4603149999998</v>
       </c>
@@ -8603,7 +10320,7 @@
         <v>8.6372664650393496</v>
       </c>
     </row>
-    <row r="69" spans="1:21">
+    <row r="69" spans="1:20">
       <c r="A69">
         <v>5059.7908310000003</v>
       </c>
@@ -8664,7 +10381,7 @@
         <v>9.0259201542189853</v>
       </c>
     </row>
-    <row r="70" spans="1:21">
+    <row r="70" spans="1:20">
       <c r="A70">
         <v>6369.7354210000003</v>
       </c>
@@ -8725,7 +10442,7 @@
         <v>0.27525042113337722</v>
       </c>
     </row>
-    <row r="71" spans="1:21">
+    <row r="71" spans="1:20">
       <c r="A71">
         <v>8019.2636849999999</v>
       </c>
@@ -8786,7 +10503,7 @@
         <v>14.094008333994923</v>
       </c>
     </row>
-    <row r="72" spans="1:21">
+    <row r="72" spans="1:20">
       <c r="A72">
         <v>10096.471541000001</v>
       </c>
@@ -8847,7 +10564,7 @@
         <v>9.2039599349631533</v>
       </c>
     </row>
-    <row r="73" spans="1:21">
+    <row r="73" spans="1:20">
       <c r="A73">
         <v>12710.556156000001</v>
       </c>
@@ -8908,7 +10625,7 @@
         <v>0.45046588130881632</v>
       </c>
     </row>
-    <row r="74" spans="1:21">
+    <row r="74" spans="1:20">
       <c r="A74">
         <v>16000.960204000001</v>
       </c>
@@ -8969,7 +10686,7 @@
         <v>5.587026360166333</v>
       </c>
     </row>
-    <row r="75" spans="1:21">
+    <row r="75" spans="1:20">
       <c r="A75" t="s">
         <v>22</v>
       </c>
@@ -8983,62 +10700,67 @@
         <v>23</v>
       </c>
     </row>
-    <row r="78" spans="1:21">
-      <c r="I78" t="s">
+    <row r="78" spans="1:20">
+      <c r="I78" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J78" t="s">
+      <c r="J78" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="N78" t="s">
+      <c r="K78" s="1"/>
+      <c r="L78" s="1"/>
+      <c r="M78" s="1"/>
+      <c r="N78" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="R78" t="s">
+      <c r="O78" s="1"/>
+      <c r="P78" s="1"/>
+      <c r="Q78" s="1"/>
+      <c r="R78" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="79" spans="1:21">
-      <c r="I79" t="s">
+      <c r="S78" s="1"/>
+      <c r="T78" s="1"/>
+    </row>
+    <row r="79" spans="1:20">
+      <c r="I79" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J79" t="s">
+      <c r="J79" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="K79" t="s">
+      <c r="K79" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="L79" t="s">
+      <c r="L79" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M79" t="s">
+      <c r="M79" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N79" t="s">
+      <c r="N79" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="O79" t="s">
+      <c r="O79" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="P79" t="s">
+      <c r="P79" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Q79" t="s">
+      <c r="Q79" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="R79" t="s">
+      <c r="R79" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="S79" t="s">
-        <v>27</v>
-      </c>
-      <c r="T79" t="s">
+      <c r="S79" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="U79" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="80" spans="1:21">
+      <c r="T79" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20">
       <c r="I80">
         <v>16.001450999999999</v>
       </c>
@@ -9051,7 +10773,7 @@
         <v>-0.00001182094500616+0.0000371505079805498i</v>
       </c>
       <c r="L80" t="str">
-        <f t="shared" ref="K80:M80" si="10">IMDIV(L44,L13)</f>
+        <f t="shared" ref="L80" si="10">IMDIV(L44,L13)</f>
         <v>1.15771682782114+0.33094514073648i</v>
       </c>
       <c r="M80" t="str">
@@ -9078,9 +10800,13 @@
         <f>DEGREES(IMARGUMENT(J80))</f>
         <v>15.207287010747224</v>
       </c>
+      <c r="S80">
+        <f t="shared" ref="S80:S110" si="12">DEGREES(IMARGUMENT(L80))</f>
+        <v>15.953123849937768</v>
+      </c>
       <c r="T80">
-        <f t="shared" ref="S80:U95" si="12">DEGREES(IMARGUMENT(L80))</f>
-        <v>15.953123849937768</v>
+        <f>N80-P80</f>
+        <v>3.1428292528697277E-2</v>
       </c>
     </row>
     <row r="81" spans="9:20">
@@ -9088,7 +10814,7 @@
         <v>20.143118000000001</v>
       </c>
       <c r="J81" t="str">
-        <f t="shared" ref="J81:M81" si="13">IMDIV(J45,J14)</f>
+        <f t="shared" ref="J81:L81" si="13">IMDIV(J45,J14)</f>
         <v>1.18982497634402+0.255306844243523i</v>
       </c>
       <c r="K81" t="str">
@@ -9123,9 +10849,13 @@
         <f t="shared" ref="R81:R110" si="19">DEGREES(IMARGUMENT(J81))</f>
         <v>12.110610214295802</v>
       </c>
-      <c r="T81">
+      <c r="S81">
         <f t="shared" si="12"/>
         <v>12.713832208061401</v>
+      </c>
+      <c r="T81">
+        <f t="shared" ref="T81:T110" si="20">N81-P81</f>
+        <v>2.4190798647864442E-2</v>
       </c>
     </row>
     <row r="82" spans="9:20">
@@ -9133,7 +10863,7 @@
         <v>25.362767999999999</v>
       </c>
       <c r="J82" t="str">
-        <f t="shared" ref="J82:M82" si="20">IMDIV(J46,J15)</f>
+        <f t="shared" ref="J82:L82" si="21">IMDIV(J46,J15)</f>
         <v>1.20526272978361+0.204653371242213i</v>
       </c>
       <c r="K82" t="str">
@@ -9141,7 +10871,7 @@
         <v>0.0000172144972262542-0.0000433612971810297i</v>
       </c>
       <c r="L82" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1.20091543846743+0.21417321831857i</v>
       </c>
       <c r="M82" t="str">
@@ -9168,9 +10898,13 @@
         <f t="shared" si="19"/>
         <v>9.6368965578238068</v>
       </c>
-      <c r="T82">
+      <c r="S82">
         <f t="shared" si="12"/>
         <v>10.111911606053829</v>
+      </c>
+      <c r="T82">
+        <f t="shared" si="20"/>
+        <v>1.8851118943758349E-2</v>
       </c>
     </row>
     <row r="83" spans="9:20">
@@ -9178,7 +10912,7 @@
         <v>31.929302</v>
       </c>
       <c r="J83" t="str">
-        <f t="shared" ref="J83:M83" si="21">IMDIV(J47,J16)</f>
+        <f t="shared" ref="J83:L83" si="22">IMDIV(J47,J16)</f>
         <v>1.21504237864512+0.163538121781689i</v>
       </c>
       <c r="K83" t="str">
@@ -9186,7 +10920,7 @@
         <v>0.0000894716219905836-0.00039594448176042i</v>
       </c>
       <c r="L83" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>1.21155606406143+0.17100948301901i</v>
       </c>
       <c r="M83" t="str">
@@ -9213,9 +10947,13 @@
         <f t="shared" si="19"/>
         <v>7.6656336040615933</v>
       </c>
-      <c r="T83">
+      <c r="S83">
         <f t="shared" si="12"/>
         <v>8.0341469320198389</v>
+      </c>
+      <c r="T83">
+        <f t="shared" si="20"/>
+        <v>1.7255966731295258E-2</v>
       </c>
     </row>
     <row r="84" spans="9:20">
@@ -9223,7 +10961,7 @@
         <v>40.195312000000001</v>
       </c>
       <c r="J84" t="str">
-        <f t="shared" ref="J84:M84" si="22">IMDIV(J48,J17)</f>
+        <f t="shared" ref="J84:L84" si="23">IMDIV(J48,J17)</f>
         <v>1.22134983408827+0.130454822926306i</v>
       </c>
       <c r="K84" t="str">
@@ -9231,7 +10969,7 @@
         <v>-0.000162915762760132-0.000030216744224611i</v>
       </c>
       <c r="L84" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>1.21843850532414+0.136384962490135i</v>
       </c>
       <c r="M84" t="str">
@@ -9258,9 +10996,13 @@
         <f t="shared" si="19"/>
         <v>6.096761544089226</v>
       </c>
-      <c r="T84">
+      <c r="S84">
         <f t="shared" si="12"/>
         <v>6.3867730060610155</v>
+      </c>
+      <c r="T84">
+        <f t="shared" si="20"/>
+        <v>1.5920685526586542E-2</v>
       </c>
     </row>
     <row r="85" spans="9:20">
@@ -9268,7 +11010,7 @@
         <v>50.597405000000002</v>
       </c>
       <c r="J85" t="str">
-        <f t="shared" ref="J85:M85" si="23">IMDIV(J49,J18)</f>
+        <f t="shared" ref="J85:L85" si="24">IMDIV(J49,J18)</f>
         <v>1.22552048837013+0.104022046133762i</v>
       </c>
       <c r="K85" t="str">
@@ -9276,7 +11018,7 @@
         <v>-0.000114389164569111+0.0000439389520602538i</v>
       </c>
       <c r="L85" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>1.22318892261629+0.108346524244376i</v>
       </c>
       <c r="M85" t="str">
@@ -9303,9 +11045,13 @@
         <f t="shared" si="19"/>
         <v>4.8516305056979325</v>
       </c>
-      <c r="T85">
+      <c r="S85">
         <f t="shared" si="12"/>
         <v>5.0618830762708447</v>
+      </c>
+      <c r="T85">
+        <f t="shared" si="20"/>
+        <v>1.3776381810493232E-2</v>
       </c>
     </row>
     <row r="86" spans="9:20">
@@ -9313,7 +11059,7 @@
         <v>63.69847</v>
       </c>
       <c r="J86" t="str">
-        <f t="shared" ref="J86:M86" si="24">IMDIV(J50,J19)</f>
+        <f t="shared" ref="J86:L86" si="25">IMDIV(J50,J19)</f>
         <v>1.22823840819385+0.0825986237504418i</v>
       </c>
       <c r="K86" t="str">
@@ -9321,7 +11067,7 @@
         <v>-0.0000146584660096872-2.75775041911732E-06i</v>
       </c>
       <c r="L86" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>1.2257172704991+0.0862682473349907i</v>
       </c>
       <c r="M86" t="str">
@@ -9348,9 +11094,13 @@
         <f t="shared" si="19"/>
         <v>3.8473291902708979</v>
       </c>
-      <c r="T86">
+      <c r="S86">
         <f t="shared" si="12"/>
         <v>4.0259439916655744</v>
+      </c>
+      <c r="T86">
+        <f t="shared" si="20"/>
+        <v>1.5984015233894366E-2</v>
       </c>
     </row>
     <row r="87" spans="9:20">
@@ -9358,7 +11108,7 @@
         <v>80.201261000000002</v>
       </c>
       <c r="J87" t="str">
-        <f t="shared" ref="J87:M87" si="25">IMDIV(J51,J20)</f>
+        <f t="shared" ref="J87:L87" si="26">IMDIV(J51,J20)</f>
         <v>1.23007368462787+0.0655618692245916i</v>
       </c>
       <c r="K87" t="str">
@@ -9366,7 +11116,7 @@
         <v>-0.0000024514057236371+5.55793065196573E-06i</v>
       </c>
       <c r="L87" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>1.2275136721214+0.0685643616130286i</v>
       </c>
       <c r="M87" t="str">
@@ -9393,9 +11143,13 @@
         <f t="shared" si="19"/>
         <v>3.0509289203341758</v>
       </c>
-      <c r="T87">
+      <c r="S87">
         <f t="shared" si="12"/>
         <v>3.1970077211597312</v>
+      </c>
+      <c r="T87">
+        <f t="shared" si="20"/>
+        <v>1.6887160391652722E-2</v>
       </c>
     </row>
     <row r="88" spans="9:20">
@@ -9403,7 +11157,7 @@
         <v>100.96802700000001</v>
       </c>
       <c r="J88" t="str">
-        <f t="shared" ref="J88:M88" si="26">IMDIV(J52,J21)</f>
+        <f t="shared" ref="J88:L88" si="27">IMDIV(J52,J21)</f>
         <v>1.2312054822528+0.0519232480296105i</v>
       </c>
       <c r="K88" t="str">
@@ -9411,7 +11165,7 @@
         <v>-0.0000534515674559565+0.0000578117589497738i</v>
       </c>
       <c r="L88" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>1.22867176733331+0.0543717973581822i</v>
       </c>
       <c r="M88" t="str">
@@ -9438,9 +11192,13 @@
         <f t="shared" si="19"/>
         <v>2.4148862140794778</v>
       </c>
-      <c r="T88">
+      <c r="S88">
         <f t="shared" si="12"/>
         <v>2.5338283595725768</v>
+      </c>
+      <c r="T88">
+        <f t="shared" si="20"/>
+        <v>1.7114051581226919E-2</v>
       </c>
     </row>
     <row r="89" spans="9:20">
@@ -9448,7 +11206,7 @@
         <v>127.10439</v>
       </c>
       <c r="J89" t="str">
-        <f t="shared" ref="J89:M89" si="27">IMDIV(J53,J22)</f>
+        <f t="shared" ref="J89:L89" si="28">IMDIV(J53,J22)</f>
         <v>1.2320832766463+0.0408715368905659i</v>
       </c>
       <c r="K89" t="str">
@@ -9456,7 +11214,7 @@
         <v>1.45245828001017E-06-2.80713218387471E-06i</v>
       </c>
       <c r="L89" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>1.22954352731884+0.0431043299427464i</v>
       </c>
       <c r="M89" t="str">
@@ -9483,9 +11241,13 @@
         <f t="shared" si="19"/>
         <v>1.8999593573984477</v>
       </c>
-      <c r="T89">
+      <c r="S89">
         <f t="shared" si="12"/>
         <v>2.0078062451108449</v>
+      </c>
+      <c r="T89">
+        <f t="shared" si="20"/>
+        <v>1.7365343504391451E-2</v>
       </c>
     </row>
     <row r="90" spans="9:20">
@@ -9493,7 +11255,7 @@
         <v>160.00702200000001</v>
       </c>
       <c r="J90" t="str">
-        <f t="shared" ref="J90:M90" si="28">IMDIV(J54,J23)</f>
+        <f t="shared" ref="J90:L90" si="29">IMDIV(J54,J23)</f>
         <v>1.23265458577318+0.0320014934703802i</v>
       </c>
       <c r="K90" t="str">
@@ -9501,7 +11263,7 @@
         <v>0.0000022662006216855-0.0000053474763750342i</v>
       </c>
       <c r="L90" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>1.23013575395005+0.0340403246805903i</v>
       </c>
       <c r="M90" t="str">
@@ -9528,9 +11290,13 @@
         <f t="shared" si="19"/>
         <v>1.4871471424604255</v>
       </c>
-      <c r="T90">
+      <c r="S90">
         <f t="shared" si="12"/>
         <v>1.5850846828597729</v>
+      </c>
+      <c r="T90">
+        <f t="shared" si="20"/>
+        <v>1.7368935461611335E-2</v>
       </c>
     </row>
     <row r="91" spans="9:20">
@@ -9538,7 +11304,7 @@
         <v>201.45634899999999</v>
       </c>
       <c r="J91" t="str">
-        <f t="shared" ref="J91:M91" si="29">IMDIV(J55,J24)</f>
+        <f t="shared" ref="J91:L91" si="30">IMDIV(J55,J24)</f>
         <v>1.23308887848666+0.0247700697676603i</v>
       </c>
       <c r="K91" t="str">
@@ -9546,7 +11312,7 @@
         <v>-4.99499383207763E-06-4.97672192683103E-06i</v>
       </c>
       <c r="L91" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>1.23064060952971+0.0267235290739473i</v>
       </c>
       <c r="M91" t="str">
@@ -9573,9 +11339,13 @@
         <f t="shared" si="19"/>
         <v>1.1507926411489813</v>
       </c>
-      <c r="T91">
+      <c r="S91">
         <f t="shared" si="12"/>
         <v>1.2439901761347154</v>
+      </c>
+      <c r="T91">
+        <f t="shared" si="20"/>
+        <v>1.6967466161546652E-2</v>
       </c>
     </row>
     <row r="92" spans="9:20">
@@ -9583,7 +11353,7 @@
         <v>253.58521099999999</v>
       </c>
       <c r="J92" t="str">
-        <f t="shared" ref="J92:M92" si="30">IMDIV(J56,J25)</f>
+        <f t="shared" ref="J92:L92" si="31">IMDIV(J56,J25)</f>
         <v>1.23330913945384+0.0188617914529088i</v>
       </c>
       <c r="K92" t="str">
@@ -9591,7 +11361,7 @@
         <v>0.0000041242453495014-1.17751068213635E-06i</v>
       </c>
       <c r="L92" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>1.23096199400956+0.0207854023968791i</v>
       </c>
       <c r="M92" t="str">
@@ -9618,9 +11388,13 @@
         <f t="shared" si="19"/>
         <v>0.87619297100963001</v>
       </c>
-      <c r="T92">
+      <c r="S92">
         <f t="shared" si="12"/>
         <v>0.96737565689332938</v>
+      </c>
+      <c r="T92">
+        <f t="shared" si="20"/>
+        <v>1.6323704568577568E-2</v>
       </c>
     </row>
     <row r="93" spans="9:20">
@@ -9628,7 +11402,7 @@
         <v>319.290075</v>
       </c>
       <c r="J93" t="str">
-        <f t="shared" ref="J93:M93" si="31">IMDIV(J57,J26)</f>
+        <f t="shared" ref="J93:L93" si="32">IMDIV(J57,J26)</f>
         <v>1.23338451032511+0.0139634716503514i</v>
       </c>
       <c r="K93" t="str">
@@ -9636,7 +11410,7 @@
         <v>-5.29970193853498E-06+4.54324743766298E-07i</v>
       </c>
       <c r="L93" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>1.23116688916065+0.015954070663567i</v>
       </c>
       <c r="M93" t="str">
@@ -9663,9 +11437,13 @@
         <f t="shared" si="19"/>
         <v>0.64863293470785166</v>
       </c>
-      <c r="T93">
+      <c r="S93">
         <f t="shared" si="12"/>
         <v>0.74242554945898798</v>
+      </c>
+      <c r="T93">
+        <f t="shared" si="20"/>
+        <v>1.5458643383487569E-2</v>
       </c>
     </row>
     <row r="94" spans="9:20">
@@ -9673,7 +11451,7 @@
         <v>401.94414</v>
       </c>
       <c r="J94" t="str">
-        <f t="shared" ref="J94:M94" si="32">IMDIV(J58,J27)</f>
+        <f t="shared" ref="J94:L94" si="33">IMDIV(J58,J27)</f>
         <v>1.2334074201538+0.0098275715121715i</v>
       </c>
       <c r="K94" t="str">
@@ -9681,7 +11459,7 @@
         <v>1.47790364092875E-06-2.20132800565757E-06i</v>
       </c>
       <c r="L94" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>1.23131624081887+0.0119582504097423i</v>
       </c>
       <c r="M94" t="str">
@@ -9708,9 +11486,13 @@
         <f t="shared" si="19"/>
         <v>0.45651294605691217</v>
       </c>
-      <c r="T94">
+      <c r="S94">
         <f t="shared" si="12"/>
         <v>0.55642548711956163</v>
+      </c>
+      <c r="T94">
+        <f t="shared" si="20"/>
+        <v>1.4605089073649324E-2</v>
       </c>
     </row>
     <row r="95" spans="9:20">
@@ -9718,7 +11500,7 @@
         <v>506.01529900000003</v>
       </c>
       <c r="J95" t="str">
-        <f t="shared" ref="J95:M95" si="33">IMDIV(J59,J28)</f>
+        <f t="shared" ref="J95:L95" si="34">IMDIV(J59,J28)</f>
         <v>1.23312269625297+0.00631080849796181i</v>
       </c>
       <c r="K95" t="str">
@@ -9726,7 +11508,7 @@
         <v>-2.86652755293367E-06-0.0000012445229984658i</v>
       </c>
       <c r="L95" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>1.23132629969545+0.00865124682363737i</v>
       </c>
       <c r="M95" t="str">
@@ -9753,9 +11535,13 @@
         <f t="shared" si="19"/>
         <v>0.29322267493784637</v>
       </c>
-      <c r="T95">
+      <c r="S95">
         <f t="shared" si="12"/>
         <v>0.40255111469836641</v>
+      </c>
+      <c r="T95">
+        <f t="shared" si="20"/>
+        <v>1.2562078638783891E-2</v>
       </c>
     </row>
     <row r="96" spans="9:20">
@@ -9763,7 +11549,7 @@
         <v>636.97722999999996</v>
       </c>
       <c r="J96" t="str">
-        <f t="shared" ref="J96:M96" si="34">IMDIV(J60,J29)</f>
+        <f t="shared" ref="J96:L96" si="35">IMDIV(J60,J29)</f>
         <v>1.23282429003413+0.00331507674914652i</v>
       </c>
       <c r="K96" t="str">
@@ -9771,7 +11557,7 @@
         <v>1.20624380546548E-06-6.85245951582045E-07i</v>
       </c>
       <c r="L96" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>1.23125276871812+0.00590118124394243i</v>
       </c>
       <c r="M96" t="str">
@@ -9798,9 +11584,13 @@
         <f t="shared" si="19"/>
         <v>0.15406854830915948</v>
       </c>
+      <c r="S96">
+        <f t="shared" si="12"/>
+        <v>0.27460664381413308</v>
+      </c>
       <c r="T96">
-        <f t="shared" ref="T96:T110" si="35">DEGREES(IMARGUMENT(L96))</f>
-        <v>0.27460664381413308</v>
+        <f t="shared" si="20"/>
+        <v>1.1010891029518355E-2</v>
       </c>
     </row>
     <row r="97" spans="9:20">
@@ -9808,7 +11598,7 @@
         <v>801.91144499999996</v>
       </c>
       <c r="J97" t="str">
-        <f t="shared" ref="J97:M97" si="36">IMDIV(J61,J30)</f>
+        <f t="shared" ref="J97:L97" si="36">IMDIV(J61,J30)</f>
         <v>1.2321027301871+0.000679105288653136i</v>
       </c>
       <c r="K97" t="str">
@@ -9843,9 +11633,13 @@
         <f t="shared" si="19"/>
         <v>3.1580047662685379E-2</v>
       </c>
+      <c r="S97">
+        <f t="shared" si="12"/>
+        <v>0.16706651012607959</v>
+      </c>
       <c r="T97">
-        <f t="shared" si="35"/>
-        <v>0.16706651012607959</v>
+        <f t="shared" si="20"/>
+        <v>8.0686624598069745E-3</v>
       </c>
     </row>
     <row r="98" spans="9:20">
@@ -9853,7 +11647,7 @@
         <v>1009.546788</v>
       </c>
       <c r="J98" t="str">
-        <f t="shared" ref="J98:M98" si="37">IMDIV(J62,J31)</f>
+        <f t="shared" ref="J98:L98" si="37">IMDIV(J62,J31)</f>
         <v>1.23144749452326-0.00157336197303679i</v>
       </c>
       <c r="K98" t="str">
@@ -9888,9 +11682,13 @@
         <f t="shared" si="19"/>
         <v>-7.3204056243149976E-2</v>
       </c>
+      <c r="S98">
+        <f t="shared" si="12"/>
+        <v>7.4946786071268243E-2</v>
+      </c>
       <c r="T98">
-        <f t="shared" si="35"/>
-        <v>7.4946786071268243E-2</v>
+        <f t="shared" si="20"/>
+        <v>5.0544687767157814E-3</v>
       </c>
     </row>
     <row r="99" spans="9:20">
@@ -9898,7 +11696,7 @@
         <v>1271.06546</v>
       </c>
       <c r="J99" t="str">
-        <f t="shared" ref="J99:M99" si="38">IMDIV(J63,J32)</f>
+        <f t="shared" ref="J99:L99" si="38">IMDIV(J63,J32)</f>
         <v>1.23048604089319-0.00363932325277976i</v>
       </c>
       <c r="K99" t="str">
@@ -9933,9 +11731,13 @@
         <f t="shared" si="19"/>
         <v>-0.1694592605951846</v>
       </c>
+      <c r="S99">
+        <f t="shared" si="12"/>
+        <v>-5.0339679061021554E-3</v>
+      </c>
       <c r="T99">
-        <f t="shared" si="35"/>
-        <v>-5.0339679061021554E-3</v>
+        <f t="shared" si="20"/>
+        <v>8.8362179071244107E-4</v>
       </c>
     </row>
     <row r="100" spans="9:20">
@@ -9943,7 +11745,7 @@
         <v>1600.019278</v>
       </c>
       <c r="J100" t="str">
-        <f t="shared" ref="J100:M100" si="39">IMDIV(J64,J33)</f>
+        <f t="shared" ref="J100:L100" si="39">IMDIV(J64,J33)</f>
         <v>1.22935756537194-0.00531589863979919i</v>
       </c>
       <c r="K100" t="str">
@@ -9978,9 +11780,13 @@
         <f t="shared" si="19"/>
         <v>-0.2477527016027524</v>
       </c>
+      <c r="S100">
+        <f t="shared" si="12"/>
+        <v>-7.4241739714049432E-2</v>
+      </c>
       <c r="T100">
-        <f t="shared" si="35"/>
-        <v>-7.4241739714049432E-2</v>
+        <f t="shared" si="20"/>
+        <v>-4.4805860565044764E-3</v>
       </c>
     </row>
     <row r="101" spans="9:20">
@@ -9988,7 +11794,7 @@
         <v>2014.3138919999999</v>
       </c>
       <c r="J101" t="str">
-        <f t="shared" ref="J101:M101" si="40">IMDIV(J65,J34)</f>
+        <f t="shared" ref="J101:L101" si="40">IMDIV(J65,J34)</f>
         <v>1.22819244481249-0.00667286450375044i</v>
       </c>
       <c r="K101" t="str">
@@ -10023,9 +11829,13 @@
         <f t="shared" si="19"/>
         <v>-0.31128933671960984</v>
       </c>
+      <c r="S101">
+        <f t="shared" si="12"/>
+        <v>-0.13557885993596089</v>
+      </c>
       <c r="T101">
-        <f t="shared" si="35"/>
-        <v>-0.13557885993596089</v>
+        <f t="shared" si="20"/>
+        <v>-1.0582951640562221E-2</v>
       </c>
     </row>
     <row r="102" spans="9:20">
@@ -10033,7 +11843,7 @@
         <v>2536.1076779999999</v>
       </c>
       <c r="J102" t="str">
-        <f t="shared" ref="J102:M102" si="41">IMDIV(J66,J35)</f>
+        <f t="shared" ref="J102:L102" si="41">IMDIV(J66,J35)</f>
         <v>1.22709383317395-0.00778931688703703i</v>
       </c>
       <c r="K102" t="str">
@@ -10068,9 +11878,13 @@
         <f t="shared" si="19"/>
         <v>-0.36369589400692298</v>
       </c>
+      <c r="S102">
+        <f t="shared" si="12"/>
+        <v>-0.1962345327672462</v>
+      </c>
       <c r="T102">
-        <f t="shared" si="35"/>
-        <v>-0.1962345327672462</v>
+        <f t="shared" si="20"/>
+        <v>-1.7173474563490165E-2</v>
       </c>
     </row>
     <row r="103" spans="9:20">
@@ -10078,7 +11892,7 @@
         <v>3192.5215979999998</v>
       </c>
       <c r="J103" t="str">
-        <f t="shared" ref="J103:M103" si="42">IMDIV(J67,J36)</f>
+        <f t="shared" ref="J103:L103" si="42">IMDIV(J67,J36)</f>
         <v>1.22621785089827-0.00874648345441892i</v>
       </c>
       <c r="K103" t="str">
@@ -10113,9 +11927,13 @@
         <f t="shared" si="19"/>
         <v>-0.40867786130878259</v>
       </c>
+      <c r="S103">
+        <f t="shared" si="12"/>
+        <v>-0.25782888455936676</v>
+      </c>
       <c r="T103">
-        <f t="shared" si="35"/>
-        <v>-0.25782888455936676</v>
+        <f t="shared" si="20"/>
+        <v>-2.2596052247830567E-2</v>
       </c>
     </row>
     <row r="104" spans="9:20">
@@ -10123,7 +11941,7 @@
         <v>4019.4603149999998</v>
       </c>
       <c r="J104" t="str">
-        <f t="shared" ref="J104:M104" si="43">IMDIV(J68,J37)</f>
+        <f t="shared" ref="J104:L104" si="43">IMDIV(J68,J37)</f>
         <v>1.22520980524367-0.00970094117642679i</v>
       </c>
       <c r="K104" t="str">
@@ -10158,9 +11976,13 @@
         <f t="shared" si="19"/>
         <v>-0.45364587329927586</v>
       </c>
+      <c r="S104">
+        <f t="shared" si="12"/>
+        <v>-0.32698073454489907</v>
+      </c>
       <c r="T104">
-        <f t="shared" si="35"/>
-        <v>-0.32698073454489907</v>
+        <f t="shared" si="20"/>
+        <v>-2.9316785388928457E-2</v>
       </c>
     </row>
     <row r="105" spans="9:20">
@@ -10168,7 +11990,7 @@
         <v>5059.7908310000003</v>
       </c>
       <c r="J105" t="str">
-        <f t="shared" ref="J105:M105" si="44">IMDIV(J69,J38)</f>
+        <f t="shared" ref="J105:L105" si="44">IMDIV(J69,J38)</f>
         <v>1.22494532495518-0.0107872381383071i</v>
       </c>
       <c r="K105" t="str">
@@ -10203,9 +12025,13 @@
         <f t="shared" si="19"/>
         <v>-0.50455087990446079</v>
       </c>
+      <c r="S105">
+        <f t="shared" si="12"/>
+        <v>-0.4081341465207915</v>
+      </c>
       <c r="T105">
-        <f t="shared" si="35"/>
-        <v>-0.4081341465207915</v>
+        <f t="shared" si="20"/>
+        <v>-3.0392752811065682E-2</v>
       </c>
     </row>
     <row r="106" spans="9:20">
@@ -10213,7 +12039,7 @@
         <v>6369.7354210000003</v>
       </c>
       <c r="J106" t="str">
-        <f t="shared" ref="J106:M106" si="45">IMDIV(J70,J39)</f>
+        <f t="shared" ref="J106:L106" si="45">IMDIV(J70,J39)</f>
         <v>1.22432590576643-0.0123391927206307i</v>
       </c>
       <c r="K106" t="str">
@@ -10248,9 +12074,13 @@
         <f t="shared" si="19"/>
         <v>-0.57742773124356195</v>
       </c>
+      <c r="S106">
+        <f t="shared" si="12"/>
+        <v>-0.51261943182823111</v>
+      </c>
       <c r="T106">
-        <f t="shared" si="35"/>
-        <v>-0.51261943182823111</v>
+        <f t="shared" si="20"/>
+        <v>-3.5023572931281333E-2</v>
       </c>
     </row>
     <row r="107" spans="9:20">
@@ -10258,7 +12088,7 @@
         <v>8019.2636849999999</v>
       </c>
       <c r="J107" t="str">
-        <f t="shared" ref="J107:M107" si="46">IMDIV(J71,J40)</f>
+        <f t="shared" ref="J107:L107" si="46">IMDIV(J71,J40)</f>
         <v>1.22409754403564-0.0145410806517118i</v>
       </c>
       <c r="K107" t="str">
@@ -10293,9 +12123,13 @@
         <f t="shared" si="19"/>
         <v>-0.6805857668068257</v>
       </c>
+      <c r="S107">
+        <f t="shared" si="12"/>
+        <v>-0.64881376746088903</v>
+      </c>
       <c r="T107">
-        <f t="shared" si="35"/>
-        <v>-0.64881376746088903</v>
+        <f t="shared" si="20"/>
+        <v>-3.7237192114306428E-2</v>
       </c>
     </row>
     <row r="108" spans="9:20">
@@ -10303,7 +12137,7 @@
         <v>10096.471541000001</v>
       </c>
       <c r="J108" t="str">
-        <f t="shared" ref="J108:M108" si="47">IMDIV(J72,J41)</f>
+        <f t="shared" ref="J108:L108" si="47">IMDIV(J72,J41)</f>
         <v>1.22412305290962-0.0170030947193164i</v>
       </c>
       <c r="K108" t="str">
@@ -10338,9 +12172,13 @@
         <f t="shared" si="19"/>
         <v>-0.7957883964232304</v>
       </c>
+      <c r="S108">
+        <f t="shared" si="12"/>
+        <v>-0.79810117785488044</v>
+      </c>
       <c r="T108">
-        <f t="shared" si="35"/>
-        <v>-0.79810117785488044</v>
+        <f t="shared" si="20"/>
+        <v>-3.9052798198924155E-2</v>
       </c>
     </row>
     <row r="109" spans="9:20">
@@ -10348,7 +12186,7 @@
         <v>12710.556156000001</v>
       </c>
       <c r="J109" t="str">
-        <f t="shared" ref="J109:M109" si="48">IMDIV(J73,J42)</f>
+        <f t="shared" ref="J109:L109" si="48">IMDIV(J73,J42)</f>
         <v>1.22397816713607-0.0208086212356548i</v>
       </c>
       <c r="K109" t="str">
@@ -10383,9 +12221,13 @@
         <f t="shared" si="19"/>
         <v>-0.9739808782619096</v>
       </c>
+      <c r="S109">
+        <f t="shared" si="12"/>
+        <v>-1.0120785530040883</v>
+      </c>
       <c r="T109">
-        <f t="shared" si="35"/>
-        <v>-1.0120785530040883</v>
+        <f t="shared" si="20"/>
+        <v>-4.0647423015186535E-2</v>
       </c>
     </row>
     <row r="110" spans="9:20">
@@ -10393,7 +12235,7 @@
         <v>16000.960204000001</v>
       </c>
       <c r="J110" t="str">
-        <f t="shared" ref="J110:M110" si="49">IMDIV(J74,J43)</f>
+        <f t="shared" ref="J110:L110" si="49">IMDIV(J74,J43)</f>
         <v>1.22404695817957-0.0254327196504228i</v>
       </c>
       <c r="K110" t="str">
@@ -10428,9 +12270,64 @@
         <f t="shared" si="19"/>
         <v>-1.1902957229025357</v>
       </c>
+      <c r="S110">
+        <f t="shared" si="12"/>
+        <v>-1.267139428473298</v>
+      </c>
       <c r="T110">
-        <f t="shared" si="35"/>
-        <v>-1.267139428473298</v>
+        <f t="shared" si="20"/>
+        <v>-4.2313640984098733E-2</v>
+      </c>
+    </row>
+    <row r="112" spans="9:20">
+      <c r="M112" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N112">
+        <f>MIN(N80:N110)</f>
+        <v>1.64460791769961</v>
+      </c>
+      <c r="P112">
+        <f>MIN(P80:P110)</f>
+        <v>1.6131796251709127</v>
+      </c>
+      <c r="T112">
+        <f>MIN(T80:T110)</f>
+        <v>-4.2313640984098733E-2</v>
+      </c>
+    </row>
+    <row r="113" spans="13:20">
+      <c r="M113" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N113">
+        <f>MAX(N80:N110)</f>
+        <v>1.8225264032190687</v>
+      </c>
+      <c r="P113">
+        <f>MAX(P80:P110)</f>
+        <v>1.8078017553218149</v>
+      </c>
+      <c r="T113">
+        <f>MAX(T80:T110)</f>
+        <v>3.1428292528697277E-2</v>
+      </c>
+    </row>
+    <row r="114" spans="13:20">
+      <c r="M114" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="N114">
+        <f>N112-N113</f>
+        <v>-0.17791848551945866</v>
+      </c>
+      <c r="P114">
+        <f>P112-P113</f>
+        <v>-0.19462213015090213</v>
+      </c>
+      <c r="T114">
+        <f>T112-T113</f>
+        <v>-7.374193351279601E-2</v>
       </c>
     </row>
   </sheetData>
@@ -10443,4 +12340,1129 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="C2:J39"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="3" max="10" width="13.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:10">
+      <c r="D2" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="3:10">
+      <c r="D3" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="3:10">
+      <c r="C4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="2">
+        <f>10000000*0.00000047/9/10</f>
+        <v>5.2222222222222225E-2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="3:10">
+      <c r="C5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="2">
+        <f>0.0000022*47000</f>
+        <v>0.10340000000000001</v>
+      </c>
+      <c r="E5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="3:10">
+      <c r="C7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="3:10">
+      <c r="C8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="3:10">
+      <c r="C9">
+        <v>16.001450999999999</v>
+      </c>
+      <c r="D9" t="str">
+        <f>COMPLEX(0, 2*PI()*C9)</f>
+        <v>100.540081816754i</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" ref="E9:E39" si="0">IMDIV(1,IMSUM(1,IMDIV(1,IMPRODUCT(_t4,D9))))</f>
+        <v>0.964994547663915+0.18379355441046i</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" ref="F9:F39" si="1">IMDIV(1,IMSUM(1,IMDIV(1,IMPRODUCT(_t5,D9))))</f>
+        <v>0.990831877147911+0.0953103791591337i</v>
+      </c>
+      <c r="G9" t="str">
+        <f>IMPRODUCT(E9,F9)</f>
+        <v>0.93862992574147+0.274082508748547i</v>
+      </c>
+      <c r="H9">
+        <f>20*LOG(IMABS(G9))</f>
+        <v>-0.1947517015915472</v>
+      </c>
+      <c r="I9">
+        <f>DEGREES(IMARGUMENT(G9))</f>
+        <v>16.277948971105101</v>
+      </c>
+      <c r="J9">
+        <f>H9+1.8</f>
+        <v>1.6052482984084528</v>
+      </c>
+    </row>
+    <row r="10" spans="3:10">
+      <c r="C10">
+        <v>20.143118000000001</v>
+      </c>
+      <c r="D10" t="str">
+        <f t="shared" ref="D10:D39" si="2">COMPLEX(0, 2*PI()*C10)</f>
+        <v>126.562943058385i</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="0"/>
+        <v>0.977620696822103+0.147913724742395i</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="1"/>
+        <v>0.994194798767747+0.075970394700214i</v>
+      </c>
+      <c r="G10" t="str">
+        <f t="shared" ref="G10:G39" si="3">IMPRODUCT(E10,F10)</f>
+        <v>0.960708347897977+0.221325286009927i</v>
+      </c>
+      <c r="H10">
+        <f t="shared" ref="H10:H39" si="4">20*LOG(IMABS(G10))</f>
+        <v>-0.12358125974333362</v>
+      </c>
+      <c r="I10">
+        <f t="shared" ref="I10:I39" si="5">DEGREES(IMARGUMENT(G10))</f>
+        <v>12.97328820950548</v>
+      </c>
+      <c r="J10">
+        <f t="shared" ref="J10:J39" si="6">H10+1.8</f>
+        <v>1.6764187402566664</v>
+      </c>
+    </row>
+    <row r="11" spans="3:10">
+      <c r="C11">
+        <v>25.362767999999999</v>
+      </c>
+      <c r="D11" t="str">
+        <f t="shared" si="2"/>
+        <v>159.358971247005i</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="0"/>
+        <v>0.985766544664573+0.118451948420619i</v>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="1"/>
+        <v>0.996330479620878+0.0604653206334792i</v>
+      </c>
+      <c r="G11" t="str">
+        <f t="shared" si="3"/>
+        <v>0.974987019198957+0.177621976774843i</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="4"/>
+        <v>-7.8225087840735896E-2</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="5"/>
+        <v>10.324846577527182</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="6"/>
+        <v>1.721774912159264</v>
+      </c>
+    </row>
+    <row r="12" spans="3:10">
+      <c r="C12">
+        <v>31.929302</v>
+      </c>
+      <c r="D12" t="str">
+        <f t="shared" si="2"/>
+        <v>200.6177211949i</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="0"/>
+        <v>0.990971576653104+0.0945881119314985i</v>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="1"/>
+        <v>0.997681472540943+0.0480952377006099i</v>
+      </c>
+      <c r="G12" t="str">
+        <f t="shared" si="3"/>
+        <v>0.984124744114491+0.142029820330364i</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="4"/>
+        <v>-4.9468946810694296E-2</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="5"/>
+        <v>8.2122781626981425</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="6"/>
+        <v>1.7505310531893057</v>
+      </c>
+    </row>
+    <row r="13" spans="3:10">
+      <c r="C13">
+        <v>40.195312000000001</v>
+      </c>
+      <c r="D13" t="str">
+        <f t="shared" si="2"/>
+        <v>252.554593775899i</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="0"/>
+        <v>0.994284039404321+0.0753875877724443i</v>
+      </c>
+      <c r="F13" t="str">
+        <f t="shared" si="1"/>
+        <v>0.998535760896873+0.038237352248502i</v>
+      </c>
+      <c r="G13" t="str">
+        <f t="shared" si="3"/>
+        <v>0.98994554808539+0.113295991368304i</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="4"/>
+        <v>-3.1259089569573718E-2</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="5"/>
+        <v>6.5289059080393237</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="6"/>
+        <v>1.7687409104304264</v>
+      </c>
+    </row>
+    <row r="14" spans="3:10">
+      <c r="C14">
+        <v>50.597405000000002</v>
+      </c>
+      <c r="D14" t="str">
+        <f t="shared" si="2"/>
+        <v>317.912871677415i</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="0"/>
+        <v>0.996385066696026+0.0600155443296285i</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999075427491249+0.0303927240376169i</v>
+      </c>
+      <c r="G14" t="str">
+        <f t="shared" si="3"/>
+        <v>0.993639800578451+0.0902429119745384i</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="4"/>
+        <v>-1.97451254588017E-2</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="5"/>
+        <v>5.189397359772232</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="6"/>
+        <v>1.7802548745411984</v>
+      </c>
+    </row>
+    <row r="15" spans="3:10">
+      <c r="C15">
+        <v>63.69847</v>
+      </c>
+      <c r="D15" t="str">
+        <f t="shared" si="2"/>
+        <v>400.22929079382i</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="0"/>
+        <v>0.99771609233811+0.0477356410628594i</v>
+      </c>
+      <c r="F15" t="str">
+        <f t="shared" si="1"/>
+        <v>0.99941643710284+0.02414999692557i</v>
+      </c>
+      <c r="G15" t="str">
+        <f t="shared" si="3"/>
+        <v>0.995981046659814+0.07180262487642i</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="4"/>
+        <v>-1.2465350366131925E-2</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="5"/>
+        <v>4.1234542564179142</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="6"/>
+        <v>1.7875346496338682</v>
+      </c>
+    </row>
+    <row r="16" spans="3:10">
+      <c r="C16">
+        <v>80.201261000000002</v>
+      </c>
+      <c r="D16" t="str">
+        <f t="shared" si="2"/>
+        <v>503.919384732475i</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="0"/>
+        <v>0.998558082197021+0.0379452062325249i</v>
+      </c>
+      <c r="F16" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999631805871877+0.0191848523895007i</v>
+      </c>
+      <c r="G16" t="str">
+        <f t="shared" si="3"/>
+        <v>0.997462445794106+0.0570884244396924i</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="4"/>
+        <v>-7.8660297966015313E-3</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="5"/>
+        <v>3.2756734668524565</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="6"/>
+        <v>1.7921339702033985</v>
+      </c>
+    </row>
+    <row r="17" spans="3:10">
+      <c r="C17">
+        <v>100.96802700000001</v>
+      </c>
+      <c r="D17" t="str">
+        <f t="shared" si="2"/>
+        <v>634.400823741312i</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999089738184671+0.0301568108187294i</v>
+      </c>
+      <c r="F17" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999767656499157+0.0152410471208609i</v>
+      </c>
+      <c r="G17" t="str">
+        <f t="shared" si="3"/>
+        <v>0.998397984802542+0.0453769778573707i</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="4"/>
+        <v>-4.9641894036725649E-3</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="5"/>
+        <v>2.6022902458806163</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="6"/>
+        <v>1.7950358105963276</v>
+      </c>
+    </row>
+    <row r="18" spans="3:10">
+      <c r="C18">
+        <v>127.10439</v>
+      </c>
+      <c r="D18" t="str">
+        <f t="shared" si="2"/>
+        <v>798.620435726024i</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="0"/>
+        <v>0.99942540895738+0.0239637411051413i</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999853372847614+0.01210808212989i</v>
+      </c>
+      <c r="G18" t="str">
+        <f t="shared" si="3"/>
+        <v>0.998988711110202+0.0360613523043774i</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="4"/>
+        <v>-3.1329747104975872E-3</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="5"/>
+        <v>2.0673572452910469</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="6"/>
+        <v>1.7968670252895025</v>
+      </c>
+    </row>
+    <row r="19" spans="3:10">
+      <c r="C19">
+        <v>160.00702200000001</v>
+      </c>
+      <c r="D19" t="str">
+        <f t="shared" si="2"/>
+        <v>1005.35376967596i</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999637344762567+0.0190400556357283i</v>
+      </c>
+      <c r="F19" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999907470351129+0.00961878823628812i</v>
+      </c>
+      <c r="G19" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999361706406891+0.0286535937984223i</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="4"/>
+        <v>-1.9771470949528046E-3</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="5"/>
+        <v>1.6423286256810403</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="6"/>
+        <v>1.7980228529050473</v>
+      </c>
+    </row>
+    <row r="20" spans="3:10">
+      <c r="C20">
+        <v>201.45634899999999</v>
+      </c>
+      <c r="D20" t="str">
+        <f t="shared" si="2"/>
+        <v>1265.78757207484i</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999771193547533+0.0151246190059189i</v>
+      </c>
+      <c r="F20" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999941627013145+0.0076399986550965i</v>
+      </c>
+      <c r="G20" t="str">
+        <f t="shared" si="3"/>
+        <v>0.99959728184793+0.0227619867108399i</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="4"/>
+        <v>-1.2473255566304948E-3</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="5"/>
+        <v>1.3044657595640947</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="6"/>
+        <v>1.7987526744433695</v>
+      </c>
+    </row>
+    <row r="21" spans="3:10">
+      <c r="C21">
+        <v>253.58521099999999</v>
+      </c>
+      <c r="D21" t="str">
+        <f t="shared" si="2"/>
+        <v>1593.32287187324i</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999855582774215+0.0120165040444467i</v>
+      </c>
+      <c r="F21" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999963158666503+0.00606959440267911i</v>
+      </c>
+      <c r="G21" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999745811455553+0.0180847791891076i</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="4"/>
+        <v>-7.8724416163340608E-4</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="5"/>
+        <v>1.036331945158887</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="6"/>
+        <v>1.7992127558383666</v>
+      </c>
+    </row>
+    <row r="22" spans="3:10">
+      <c r="C22">
+        <v>319.290075</v>
+      </c>
+      <c r="D22" t="str">
+        <f t="shared" si="2"/>
+        <v>2006.15870796827i</v>
+      </c>
+      <c r="E22" t="str">
+        <f t="shared" si="0"/>
+        <v>0.99990889983524+0.00954420586114244i</v>
+      </c>
+      <c r="F22" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999976760956157+0.00482063313164626i</v>
+      </c>
+      <c r="G22" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999839653793488+0.0143641780340977i</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="4"/>
+        <v>-4.965880690104876E-4</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="5"/>
+        <v>0.82308214092545096</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="6"/>
+        <v>1.7995034119309896</v>
+      </c>
+    </row>
+    <row r="23" spans="3:10">
+      <c r="C23">
+        <v>401.94414</v>
+      </c>
+      <c r="D23" t="str">
+        <f t="shared" si="2"/>
+        <v>2525.48951475493i</v>
+      </c>
+      <c r="E23" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999942512529956+0.00758183125863281i</v>
+      </c>
+      <c r="F23" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999985335697383+0.00382937169461019i</v>
+      </c>
+      <c r="G23" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999898815420338+0.0114108716300845i</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="4"/>
+        <v>-3.1335881079754761E-4</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="5"/>
+        <v>0.65383256278141244</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="6"/>
+        <v>1.7996866411892025</v>
+      </c>
+    </row>
+    <row r="24" spans="3:10">
+      <c r="C24">
+        <v>506.01529900000003</v>
+      </c>
+      <c r="D24" t="str">
+        <f t="shared" si="2"/>
+        <v>3179.38789188489i</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999963726745958+0.00602261888990038i</v>
+      </c>
+      <c r="F24" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999990747312978+0.00304180890423274i</v>
+      </c>
+      <c r="G24" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999936154738795+0.00906426173241835i</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="4"/>
+        <v>-1.9771969296170184E-4</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="5"/>
+        <v>0.51936287616798449</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="6"/>
+        <v>1.7998022803070384</v>
+      </c>
+    </row>
+    <row r="25" spans="3:10">
+      <c r="C25">
+        <v>636.97722999999996</v>
+      </c>
+      <c r="D25" t="str">
+        <f t="shared" si="2"/>
+        <v>4002.24597254395i</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="0"/>
+        <v>0.99997710862875+0.0047844380270897i</v>
+      </c>
+      <c r="F25" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999994160860726+0.00241642404762851i</v>
+      </c>
+      <c r="G25" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999959708392039+0.00720077882245825i</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="4"/>
+        <v>-1.2477623376801639E-4</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="5"/>
+        <v>0.41258372821785916</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="6"/>
+        <v>1.7998752237662321</v>
+      </c>
+    </row>
+    <row r="26" spans="3:10">
+      <c r="C26">
+        <v>801.91144499999996</v>
+      </c>
+      <c r="D26" t="str">
+        <f t="shared" si="2"/>
+        <v>5038.55820888315i</v>
+      </c>
+      <c r="E26" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999985556565713+0.00380042440713531i</v>
+      </c>
+      <c r="F26" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999996315786734+0.00191942691784448i</v>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999974577768753+0.00571980960028922i</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="4"/>
+        <v>-7.8727855499073241E-5</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="5"/>
+        <v>0.32772570719170235</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="6"/>
+        <v>1.799921272144501</v>
+      </c>
+    </row>
+    <row r="27" spans="3:10">
+      <c r="C27">
+        <v>1009.546788</v>
+      </c>
+      <c r="D27" t="str">
+        <f t="shared" si="2"/>
+        <v>6343.16954527195i</v>
+      </c>
+      <c r="E27" t="str">
+        <f t="shared" si="0"/>
+        <v>0.99999088676214+0.00301880022672194i</v>
+      </c>
+      <c r="F27" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999997675415844+0.00152465692954447i</v>
+      </c>
+      <c r="G27" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999983959564484+0.00454343624424998i</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="4"/>
+        <v>-4.9674021940286812E-5</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="5"/>
+        <v>0.26032210568319675</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="6"/>
+        <v>1.7999503259780598</v>
+      </c>
+    </row>
+    <row r="28" spans="3:10">
+      <c r="C28">
+        <v>1271.06546</v>
+      </c>
+      <c r="D28" t="str">
+        <f t="shared" si="2"/>
+        <v>7986.33982273546i</v>
+      </c>
+      <c r="E28" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999994251014214+0.00239769738181416i</v>
+      </c>
+      <c r="F28" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999998533565349+0.00121096345966406i</v>
+      </c>
+      <c r="G28" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999989881064077+0.00360865036359998i</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="4"/>
+        <v>-3.1336249242150979E-5</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="5"/>
+        <v>0.20676163026639982</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="6"/>
+        <v>1.7999686637507579</v>
+      </c>
+    </row>
+    <row r="29" spans="3:10">
+      <c r="C29">
+        <v>1600.019278</v>
+      </c>
+      <c r="D29" t="str">
+        <f t="shared" si="2"/>
+        <v>10053.2176187337i</v>
+      </c>
+      <c r="E29" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999996371914109+0.00190475004346316i</v>
+      </c>
+      <c r="F29" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999074559816+0.000961997571387057i</v>
+      </c>
+      <c r="G29" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999993614112367+0.00286674236190817i</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="4"/>
+        <v>-1.9775742915273929E-5</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="5"/>
+        <v>0.16425283723211134</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="6"/>
+        <v>1.7999802242570848</v>
+      </c>
+    </row>
+    <row r="30" spans="3:10">
+      <c r="C30">
+        <v>2014.3138919999999</v>
+      </c>
+      <c r="D30" t="str">
+        <f t="shared" si="2"/>
+        <v>12656.3074502621i</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999997710849869+0.00151299203268221i</v>
+      </c>
+      <c r="F30" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999416091716+0.000764138693285578i</v>
+      </c>
+      <c r="G30" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999995970807167+0.00227712809329102i</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="4"/>
+        <v>-1.247754627835847E-5</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="5"/>
+        <v>0.13047012933550328</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="6"/>
+        <v>1.7999875224537216</v>
+      </c>
+    </row>
+    <row r="31" spans="3:10">
+      <c r="C31">
+        <v>2536.1076779999999</v>
+      </c>
+      <c r="D31" t="str">
+        <f t="shared" si="2"/>
+        <v>15934.8344998349i</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999998555912325+0.00120170112326353i</v>
+      </c>
+      <c r="F31" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999631647478+0.000606920412109867i</v>
+      </c>
+      <c r="G31" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999997458223394+0.00180862021627747i</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="4"/>
+        <v>-7.8713325837279372E-6</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="5"/>
+        <v>0.10362645553877131</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="6"/>
+        <v>1.7999921286674163</v>
+      </c>
+    </row>
+    <row r="32" spans="3:10">
+      <c r="C32">
+        <v>3192.5215979999998</v>
+      </c>
+      <c r="D32" t="str">
+        <f t="shared" si="2"/>
+        <v>20059.2047974071i</v>
+      </c>
+      <c r="E32" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999999088699765+0.000954620031710228i</v>
+      </c>
+      <c r="F32" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999767549012+0.000482131656441369i</v>
+      </c>
+      <c r="G32" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999998395996452+0.00143675102688254i</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="4"/>
+        <v>-4.967250362532777E-6</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="5"/>
+        <v>8.2319845449711063E-2</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="6"/>
+        <v>1.7999950327496375</v>
+      </c>
+    </row>
+    <row r="33" spans="3:10">
+      <c r="C33">
+        <v>4019.4603149999998</v>
+      </c>
+      <c r="D33" t="str">
+        <f t="shared" si="2"/>
+        <v>25255.0139939994i</v>
+      </c>
+      <c r="E33" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999999425097991+0.000758222710389337i</v>
+      </c>
+      <c r="F33" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999853356225+0.000382940926820527i</v>
+      </c>
+      <c r="G33" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999998988099793+0.00114116330586772i</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="4"/>
+        <v>-3.1336342873150856E-6</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="5"/>
+        <v>6.5383878941226214E-2</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="6"/>
+        <v>1.7999968663657127</v>
+      </c>
+    </row>
+    <row r="34" spans="3:10">
+      <c r="C34">
+        <v>5059.7908310000003</v>
+      </c>
+      <c r="D34" t="str">
+        <f t="shared" si="2"/>
+        <v>31791.6034067412i</v>
+      </c>
+      <c r="E34" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999999637202504+0.000602326626248937i</v>
+      </c>
+      <c r="F34" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999907459036+0.00030420544900591i</v>
+      </c>
+      <c r="G34" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999999361430532+0.000906531909149985i</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="4"/>
+        <v>-1.9775101082273817E-6</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="5"/>
+        <v>5.194047132759607E-2</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="6"/>
+        <v>1.7999980224898917</v>
+      </c>
+    </row>
+    <row r="35" spans="3:10">
+      <c r="C35">
+        <v>6369.7354210000003</v>
+      </c>
+      <c r="D35" t="str">
+        <f t="shared" si="2"/>
+        <v>40022.2280078486i</v>
+      </c>
+      <c r="E35" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999999771078449+0.000478457415785381i</v>
+      </c>
+      <c r="F35" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999941607594+0.000241645200695118i</v>
+      </c>
+      <c r="G35" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999999597069118+0.000720102533224425i</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="4"/>
+        <v>-1.2477887808149889E-6</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="5"/>
+        <v>4.1258845463340563E-2</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="6"/>
+        <v>1.7999987522112193</v>
+      </c>
+    </row>
+    <row r="36" spans="3:10">
+      <c r="C36">
+        <v>8019.2636849999999</v>
+      </c>
+      <c r="D36" t="str">
+        <f t="shared" si="2"/>
+        <v>50386.5197599908i</v>
+      </c>
+      <c r="E36" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999999855568968+0.000380040802494903i</v>
+      </c>
+      <c r="F36" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999963159104+0.000191939819890682i</v>
+      </c>
+      <c r="G36" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999999745783114+0.000571980580662475i</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="4"/>
+        <v>-7.872540293414922E-7</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="5"/>
+        <v>3.277207799269314E-2</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="6"/>
+        <v>1.7999992127459707</v>
+      </c>
+    </row>
+    <row r="37" spans="3:10">
+      <c r="C37">
+        <v>10096.471541000001</v>
+      </c>
+      <c r="D37" t="str">
+        <f t="shared" si="2"/>
+        <v>63438.001640768i</v>
+      </c>
+      <c r="E37" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999999908884917+0.000301852737005983i</v>
+      </c>
+      <c r="F37" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999976758726+0.000152450887623172i</v>
+      </c>
+      <c r="G37" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999999839625927+0.000454303603723138i</v>
+      </c>
+      <c r="H37">
+        <f t="shared" si="4"/>
+        <v>-4.9664337125335468E-7</v>
+      </c>
+      <c r="I37">
+        <f t="shared" si="5"/>
+        <v>2.602968149463486E-2</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="6"/>
+        <v>1.7999995033566287</v>
+      </c>
+    </row>
+    <row r="38" spans="3:10">
+      <c r="C38">
+        <v>12710.556156000001</v>
+      </c>
+      <c r="D38" t="str">
+        <f t="shared" si="2"/>
+        <v>79862.7796854602i</v>
+      </c>
+      <c r="E38" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999999942508924+0.000239772959878656i</v>
+      </c>
+      <c r="F38" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999985335405+0.000121097459670348i</v>
+      </c>
+      <c r="G38" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999999898808434+0.000360870409070807i</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="4"/>
+        <v>-3.1336810315882668E-7</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="5"/>
+        <v>2.0676352585646315E-2</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="6"/>
+        <v>1.7999996866318968</v>
+      </c>
+    </row>
+    <row r="39" spans="3:10">
+      <c r="C39">
+        <v>16000.960204000001</v>
+      </c>
+      <c r="D39" t="str">
+        <f t="shared" si="2"/>
+        <v>100536.998054538i</v>
+      </c>
+      <c r="E39" t="str">
+        <f t="shared" si="0"/>
+        <v>0.999999963722491+0.000190466553070835i</v>
+      </c>
+      <c r="F39" t="str">
+        <f t="shared" si="1"/>
+        <v>0.999999990746477+0.0000961952314232327i</v>
+      </c>
+      <c r="G39" t="str">
+        <f t="shared" si="3"/>
+        <v>0.999999936146994+0.000286661779241858i</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="4"/>
+        <v>-1.9773876491545059E-7</v>
+      </c>
+      <c r="I39">
+        <f t="shared" si="5"/>
+        <v>1.6424510697129146E-2</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="6"/>
+        <v>1.7999998022612351</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>